<commit_message>
Telemetry added United Sep 29
</commit_message>
<xml_diff>
--- a/EquipAI/TestData/JCB_07_26_new_correct.xlsx
+++ b/EquipAI/TestData/JCB_07_26_new_correct.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EquipAI\Test Data\Telemetry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cursor Projects\EquipAI\EquipAI\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E670200-6215-4C8B-9D7B-466ED97F77C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78EB5138-A078-4EA9-9EA7-AB849D213B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="79">
   <si>
     <t>Account Name</t>
   </si>
@@ -263,228 +263,6 @@
   <si>
     <t>40.5709080, -112.0619000</t>
   </si>
-  <si>
-    <t>460-1060</t>
-  </si>
-  <si>
-    <t>TELEHANDLER 10000LB 42-44FT LIFT ROPS</t>
-  </si>
-  <si>
-    <t>JLG</t>
-  </si>
-  <si>
-    <t>06/28/2026 05:00 AM</t>
-  </si>
-  <si>
-    <t>PERRY WASTEWATER PLANT</t>
-  </si>
-  <si>
-    <t>1 - PROPERTY</t>
-  </si>
-  <si>
-    <t>1061-4401</t>
-  </si>
-  <si>
-    <t>ALEX RODRIGUEZ</t>
-  </si>
-  <si>
-    <t>06/04/2026 12:20 PM</t>
-  </si>
-  <si>
-    <t>32.4325250, -83.6114780</t>
-  </si>
-  <si>
-    <t>KUBOTA</t>
-  </si>
-  <si>
-    <t>RTV-X1140WH</t>
-  </si>
-  <si>
-    <t>A5KD2GDBKPG061135</t>
-  </si>
-  <si>
-    <t>32.4119570, -90.1914780</t>
-  </si>
-  <si>
-    <t>501-1100</t>
-  </si>
-  <si>
-    <t>100KW GENERATOR DSL</t>
-  </si>
-  <si>
-    <t>MULTIQUIP</t>
-  </si>
-  <si>
-    <t>DCA125SSIU4F</t>
-  </si>
-  <si>
-    <t>06/22/2026 09:00 AM</t>
-  </si>
-  <si>
-    <t>PROJECT POWEHOUSE WAREHOUSE</t>
-  </si>
-  <si>
-    <t>1 - PROJECT POWEHOUS</t>
-  </si>
-  <si>
-    <t>PROJECT POWERHOUSE</t>
-  </si>
-  <si>
-    <t>TERRELL WOODS</t>
-  </si>
-  <si>
-    <t>06/04/2026 12:13 PM</t>
-  </si>
-  <si>
-    <t>30.6439800, -96.4836270</t>
-  </si>
-  <si>
-    <t>A5KD2GDBTRG068750</t>
-  </si>
-  <si>
-    <t>06/04/2026 12:16 PM</t>
-  </si>
-  <si>
-    <t>32.4122000, -90.1859370</t>
-  </si>
-  <si>
-    <t>460-1085</t>
-  </si>
-  <si>
-    <t>TELEHANDLER 12000LB 55-56FT LIFT CAB</t>
-  </si>
-  <si>
-    <t>SANY</t>
-  </si>
-  <si>
-    <t>STH1256</t>
-  </si>
-  <si>
-    <t>TH1256CD1743</t>
-  </si>
-  <si>
-    <t>06/18/2026 05:00 AM</t>
-  </si>
-  <si>
-    <t>PO#6704207001</t>
-  </si>
-  <si>
-    <t>REYNOLDS,VERN</t>
-  </si>
-  <si>
-    <t>06/04/2026 12:27 PM</t>
-  </si>
-  <si>
-    <t>40.7984820, -111.9058400</t>
-  </si>
-  <si>
-    <t>A5KD2GDBTRG074757</t>
-  </si>
-  <si>
-    <t>32.4045250, -90.1873350</t>
-  </si>
-  <si>
-    <t>410-2020</t>
-  </si>
-  <si>
-    <t>BOOM ARTICULATED 30FT NAR ROT JIB ELEC</t>
-  </si>
-  <si>
-    <t>E300AJP</t>
-  </si>
-  <si>
-    <t>914B</t>
-  </si>
-  <si>
-    <t>06/04/2026 04:00 AM</t>
-  </si>
-  <si>
-    <t>DIAGEO MONTGOMERY BEVERAGE</t>
-  </si>
-  <si>
-    <t>1 - DIAGEO MONTGOMER</t>
-  </si>
-  <si>
-    <t>TOMA, RONNIE</t>
-  </si>
-  <si>
-    <t>32.2799080, -86.3634600</t>
-  </si>
-  <si>
-    <t>460-1030</t>
-  </si>
-  <si>
-    <t>TELEHANDLER 6000LB 42-44FT LIFT ROPS</t>
-  </si>
-  <si>
-    <t>SKYTRAK</t>
-  </si>
-  <si>
-    <t>06/12/2026 04:00 AM</t>
-  </si>
-  <si>
-    <t>WATER TREATMENT PLANT</t>
-  </si>
-  <si>
-    <t>1 - WATER TREATMENT</t>
-  </si>
-  <si>
-    <t>1061-5300</t>
-  </si>
-  <si>
-    <t>STEVEN KELLEY</t>
-  </si>
-  <si>
-    <t>06/04/2026 12:14 PM</t>
-  </si>
-  <si>
-    <t>26.7718030, -82.0350630</t>
-  </si>
-  <si>
-    <t>630-1265</t>
-  </si>
-  <si>
-    <t>CART UTV 4 PASSENGER GAS WITH CAB</t>
-  </si>
-  <si>
-    <t>XP1000 NORTHSTA</t>
-  </si>
-  <si>
-    <t>4XARS3998S8774853</t>
-  </si>
-  <si>
-    <t>06/04/2026 12:18 PM</t>
-  </si>
-  <si>
-    <t>32.4040580, -90.1865220</t>
-  </si>
-  <si>
-    <t>4XARS3991S8776153</t>
-  </si>
-  <si>
-    <t>06/26/2026 04:00 AM</t>
-  </si>
-  <si>
-    <t>JEFF,DOWNS</t>
-  </si>
-  <si>
-    <t>32.4039300, -90.1873900</t>
-  </si>
-  <si>
-    <t>4XARS3997S8774097</t>
-  </si>
-  <si>
-    <t>06/04/2026 12:26 PM</t>
-  </si>
-  <si>
-    <t>32.4043780, -90.1871780</t>
-  </si>
-  <si>
-    <t>4XARS3994S8774297</t>
-  </si>
-  <si>
-    <t>32.4119230, -90.1860270</t>
-  </si>
 </sst>
 </file>
 
@@ -606,10 +384,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -634,6 +408,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1000"/>
+  <dimension ref="A1:AH988"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.109375" customWidth="1"/>
@@ -895,13 +673,13 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -931,7 +709,7 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="11" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -982,7 +760,7 @@
       <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="15" t="s">
+      <c r="AF1" s="13" t="s">
         <v>31</v>
       </c>
       <c r="AG1" s="1" t="s">
@@ -999,13 +777,13 @@
       <c r="B2" s="3">
         <v>7265672</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="8">
         <v>210342678</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="10" t="s">
         <v>36</v>
       </c>
       <c r="F2" s="3">
@@ -1035,7 +813,7 @@
       <c r="N2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="12" t="s">
         <v>41</v>
       </c>
       <c r="P2" s="4" t="s">
@@ -1086,7 +864,7 @@
       <c r="AE2" s="3">
         <v>51.57</v>
       </c>
-      <c r="AF2" s="16">
+      <c r="AF2" s="14">
         <v>140.91999999999999</v>
       </c>
       <c r="AG2" s="3" t="s">
@@ -1103,13 +881,13 @@
       <c r="B3" s="3">
         <v>7265672</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>210398716</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="10" t="s">
         <v>48</v>
       </c>
       <c r="F3" s="3">
@@ -1139,7 +917,7 @@
       <c r="N3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="O3" s="14" t="s">
+      <c r="O3" s="12" t="s">
         <v>54</v>
       </c>
       <c r="P3" s="4" t="s">
@@ -1190,7 +968,7 @@
       <c r="AE3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AF3" s="16">
+      <c r="AF3" s="14">
         <v>20.64</v>
       </c>
       <c r="AG3" s="3" t="s">
@@ -1207,13 +985,13 @@
       <c r="B4" s="3">
         <v>7265672</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>210438462</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="10" t="s">
         <v>61</v>
       </c>
       <c r="F4" s="3">
@@ -1243,7 +1021,7 @@
       <c r="N4" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="O4" s="14" t="s">
+      <c r="O4" s="12" t="s">
         <v>65</v>
       </c>
       <c r="P4" s="4" t="s">
@@ -1294,7 +1072,7 @@
       <c r="AE4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AF4" s="16">
+      <c r="AF4" s="14">
         <v>96.49</v>
       </c>
       <c r="AG4" s="3" t="s">
@@ -1311,13 +1089,13 @@
       <c r="B5" s="3">
         <v>7265672</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <v>210441502</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="10" t="s">
         <v>61</v>
       </c>
       <c r="F5" s="3">
@@ -1347,7 +1125,7 @@
       <c r="N5" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="O5" s="14" t="s">
+      <c r="O5" s="12" t="s">
         <v>65</v>
       </c>
       <c r="P5" s="4" t="s">
@@ -1398,7 +1176,7 @@
       <c r="AE5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AF5" s="16" t="s">
+      <c r="AF5" s="14" t="s">
         <v>39</v>
       </c>
       <c r="AG5" s="3" t="s">
@@ -1415,13 +1193,13 @@
       <c r="B6" s="3">
         <v>7265672</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <v>800213755</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="10" t="s">
         <v>74</v>
       </c>
       <c r="F6" s="3">
@@ -1451,7 +1229,7 @@
       <c r="N6" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="O6" s="14" t="s">
+      <c r="O6" s="12" t="s">
         <v>41</v>
       </c>
       <c r="P6" s="4" t="s">
@@ -1502,7 +1280,7 @@
       <c r="AE6" s="3">
         <v>8796.76</v>
       </c>
-      <c r="AF6" s="16">
+      <c r="AF6" s="14">
         <v>138.72</v>
       </c>
       <c r="AG6" s="3" t="s">
@@ -1513,1259 +1291,443 @@
       </c>
     </row>
     <row r="7" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C7" s="10">
-        <v>800395291</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="F7" s="3">
-        <v>2023</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H7" s="3">
-        <v>10042</v>
-      </c>
-      <c r="I7" s="3">
-        <v>160120645</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K7" s="3">
-        <v>9327</v>
-      </c>
-      <c r="L7" s="4">
-        <v>34560863</v>
-      </c>
-      <c r="M7" s="3">
-        <v>45412.208333333336</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="O7" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="P7" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q7" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R7" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="S7" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="T7" s="4">
-        <v>12.9</v>
-      </c>
-      <c r="U7" s="3">
-        <v>0.81</v>
-      </c>
-      <c r="V7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W7" s="4">
-        <v>170.6</v>
-      </c>
-      <c r="X7" s="4">
-        <v>100</v>
-      </c>
-      <c r="Y7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z7" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC7" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="3">
-        <v>7339</v>
-      </c>
-      <c r="AE7" s="3">
-        <v>396.44</v>
-      </c>
-      <c r="AF7" s="16">
-        <v>1611.75</v>
-      </c>
-      <c r="AG7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH7" s="4" t="s">
-        <v>88</v>
-      </c>
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
+      <c r="AA7" s="6"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="5"/>
+      <c r="AD7" s="5"/>
+      <c r="AE7" s="5"/>
+      <c r="AF7" s="5"/>
+      <c r="AG7" s="5"/>
+      <c r="AH7" s="6"/>
     </row>
     <row r="8" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C8" s="10">
-        <v>800426051</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="3">
-        <v>2023</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L8" s="4">
-        <v>36632658</v>
-      </c>
-      <c r="M8" s="3">
-        <v>46161.166666666672</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="O8" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q8" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="R8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="S8" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="T8" s="4">
-        <v>13</v>
-      </c>
-      <c r="U8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="V8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="X8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE8" s="3">
-        <v>2510.34</v>
-      </c>
-      <c r="AF8" s="16">
-        <v>415.87</v>
-      </c>
-      <c r="AG8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH8" s="4" t="s">
-        <v>92</v>
-      </c>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="6"/>
+      <c r="W8" s="6"/>
+      <c r="X8" s="6"/>
+      <c r="Y8" s="6"/>
+      <c r="Z8" s="6"/>
+      <c r="AA8" s="6"/>
+      <c r="AB8" s="5"/>
+      <c r="AC8" s="5"/>
+      <c r="AD8" s="5"/>
+      <c r="AE8" s="5"/>
+      <c r="AF8" s="5"/>
+      <c r="AG8" s="5"/>
+      <c r="AH8" s="6"/>
     </row>
     <row r="9" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C9" s="10">
-        <v>800443474</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="F9" s="3">
-        <v>2023</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="I9" s="3">
-        <v>7514107</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K9" s="3">
-        <v>9405</v>
-      </c>
-      <c r="L9" s="4">
-        <v>36597859</v>
-      </c>
-      <c r="M9" s="3">
-        <v>46136.375</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="O9" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="P9" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q9" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="R9" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="S9" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="T9" s="4">
-        <v>14.63</v>
-      </c>
-      <c r="U9" s="3">
-        <v>0.54</v>
-      </c>
-      <c r="V9" s="4">
-        <v>33</v>
-      </c>
-      <c r="W9" s="4">
-        <v>176</v>
-      </c>
-      <c r="X9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z9" s="4">
-        <v>4</v>
-      </c>
-      <c r="AA9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD9" s="3">
-        <v>48623</v>
-      </c>
-      <c r="AE9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AF9" s="16">
-        <v>7350.85</v>
-      </c>
-      <c r="AG9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH9" s="4" t="s">
-        <v>103</v>
-      </c>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="6"/>
+      <c r="W9" s="6"/>
+      <c r="X9" s="6"/>
+      <c r="Y9" s="6"/>
+      <c r="Z9" s="6"/>
+      <c r="AA9" s="6"/>
+      <c r="AB9" s="5"/>
+      <c r="AC9" s="5"/>
+      <c r="AD9" s="5"/>
+      <c r="AE9" s="5"/>
+      <c r="AF9" s="5"/>
+      <c r="AG9" s="5"/>
+      <c r="AH9" s="6"/>
     </row>
     <row r="10" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B10" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C10" s="10">
-        <v>800451697</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="3">
-        <v>2024</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L10" s="4">
-        <v>36632658</v>
-      </c>
-      <c r="M10" s="3">
-        <v>46161.166666666672</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="O10" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="R10" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="S10" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="T10" s="4">
-        <v>13</v>
-      </c>
-      <c r="U10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="V10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="X10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE10" s="3">
-        <v>2080.9699999999998</v>
-      </c>
-      <c r="AF10" s="16">
-        <v>458.73</v>
-      </c>
-      <c r="AG10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH10" s="4" t="s">
-        <v>106</v>
-      </c>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="6"/>
+      <c r="W10" s="6"/>
+      <c r="X10" s="6"/>
+      <c r="Y10" s="6"/>
+      <c r="Z10" s="6"/>
+      <c r="AA10" s="6"/>
+      <c r="AB10" s="5"/>
+      <c r="AC10" s="5"/>
+      <c r="AD10" s="5"/>
+      <c r="AE10" s="5"/>
+      <c r="AF10" s="5"/>
+      <c r="AG10" s="5"/>
+      <c r="AH10" s="6"/>
     </row>
     <row r="11" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C11" s="10">
-        <v>800453796</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" s="3">
-        <v>2023</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K11" s="3">
-        <v>9615</v>
-      </c>
-      <c r="L11" s="4">
-        <v>35535767</v>
-      </c>
-      <c r="M11" s="3">
-        <v>45797.208333333336</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="O11" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q11" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="R11" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="S11" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="T11" s="4">
-        <v>25.7</v>
-      </c>
-      <c r="U11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="V11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="X11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE11" s="3">
-        <v>0.62</v>
-      </c>
-      <c r="AF11" s="16">
-        <v>799.38</v>
-      </c>
-      <c r="AG11" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH11" s="4" t="s">
-        <v>116</v>
-      </c>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="5"/>
+      <c r="V11" s="6"/>
+      <c r="W11" s="6"/>
+      <c r="X11" s="6"/>
+      <c r="Y11" s="6"/>
+      <c r="Z11" s="6"/>
+      <c r="AA11" s="6"/>
+      <c r="AB11" s="5"/>
+      <c r="AC11" s="5"/>
+      <c r="AD11" s="5"/>
+      <c r="AE11" s="5"/>
+      <c r="AF11" s="5"/>
+      <c r="AG11" s="5"/>
+      <c r="AH11" s="6"/>
     </row>
     <row r="12" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C12" s="10">
-        <v>800474744</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="3">
-        <v>2024</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L12" s="4">
-        <v>36632658</v>
-      </c>
-      <c r="M12" s="3">
-        <v>46161.166666666672</v>
-      </c>
-      <c r="N12" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="O12" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="P12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="R12" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="S12" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="T12" s="4">
-        <v>13.2</v>
-      </c>
-      <c r="U12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="V12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="X12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE12" s="3">
-        <v>2013.87</v>
-      </c>
-      <c r="AF12" s="16">
-        <v>683.1</v>
-      </c>
-      <c r="AG12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH12" s="4" t="s">
-        <v>118</v>
-      </c>
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="5"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="5"/>
+      <c r="V12" s="6"/>
+      <c r="W12" s="6"/>
+      <c r="X12" s="6"/>
+      <c r="Y12" s="6"/>
+      <c r="Z12" s="6"/>
+      <c r="AA12" s="6"/>
+      <c r="AB12" s="5"/>
+      <c r="AC12" s="5"/>
+      <c r="AD12" s="5"/>
+      <c r="AE12" s="5"/>
+      <c r="AF12" s="5"/>
+      <c r="AG12" s="5"/>
+      <c r="AH12" s="6"/>
     </row>
     <row r="13" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C13" s="10">
-        <v>800478541</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="F13" s="3">
-        <v>2024</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="I13" s="3">
-        <v>300321429</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="L13" s="4">
-        <v>36334741</v>
-      </c>
-      <c r="M13" s="3">
-        <v>46065.166666666672</v>
-      </c>
-      <c r="N13" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="O13" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="P13" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="Q13" s="3">
-        <v>3801146301</v>
-      </c>
-      <c r="R13" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="S13" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="T13" s="4">
-        <v>13.5</v>
-      </c>
-      <c r="U13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="V13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="X13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE13" s="3">
-        <v>1289.3499999999999</v>
-      </c>
-      <c r="AF13" s="16">
-        <v>10574.55</v>
-      </c>
-      <c r="AG13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH13" s="4" t="s">
-        <v>127</v>
-      </c>
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="5"/>
+      <c r="V13" s="6"/>
+      <c r="W13" s="6"/>
+      <c r="X13" s="6"/>
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6"/>
+      <c r="AA13" s="6"/>
+      <c r="AB13" s="5"/>
+      <c r="AC13" s="5"/>
+      <c r="AD13" s="5"/>
+      <c r="AE13" s="5"/>
+      <c r="AF13" s="5"/>
+      <c r="AG13" s="5"/>
+      <c r="AH13" s="6"/>
     </row>
     <row r="14" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C14" s="10">
-        <v>800481172</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="F14" s="3">
-        <v>2025</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="H14" s="3">
-        <v>6042</v>
-      </c>
-      <c r="I14" s="3">
-        <v>160136810</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K14" s="3">
-        <v>9282</v>
-      </c>
-      <c r="L14" s="4">
-        <v>36439358</v>
-      </c>
-      <c r="M14" s="3">
-        <v>46101.166666666672</v>
-      </c>
-      <c r="N14" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="O14" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="P14" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="Q14" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="R14" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="S14" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="T14" s="4">
-        <v>12.6</v>
-      </c>
-      <c r="U14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="V14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W14" s="4">
-        <v>183.20000000000002</v>
-      </c>
-      <c r="X14" s="4">
-        <v>100</v>
-      </c>
-      <c r="Y14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z14" s="4">
-        <v>276</v>
-      </c>
-      <c r="AA14" s="4">
-        <v>285</v>
-      </c>
-      <c r="AB14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE14" s="3">
-        <v>60.27</v>
-      </c>
-      <c r="AF14" s="16">
-        <v>268.75</v>
-      </c>
-      <c r="AG14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH14" s="4" t="s">
-        <v>137</v>
-      </c>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="5"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="5"/>
+      <c r="V14" s="6"/>
+      <c r="W14" s="6"/>
+      <c r="X14" s="6"/>
+      <c r="Y14" s="6"/>
+      <c r="Z14" s="6"/>
+      <c r="AA14" s="6"/>
+      <c r="AB14" s="5"/>
+      <c r="AC14" s="5"/>
+      <c r="AD14" s="5"/>
+      <c r="AE14" s="5"/>
+      <c r="AF14" s="5"/>
+      <c r="AG14" s="5"/>
+      <c r="AH14" s="6"/>
     </row>
     <row r="15" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C15" s="10">
-        <v>800483606</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="F15" s="3">
-        <v>2024</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L15" s="4">
-        <v>35199780</v>
-      </c>
-      <c r="M15" s="3">
-        <v>45660.166666666672</v>
-      </c>
-      <c r="N15" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="O15" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="P15" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q15" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="R15" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S15" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="T15" s="4">
-        <v>12.7</v>
-      </c>
-      <c r="U15" s="3">
-        <v>1</v>
-      </c>
-      <c r="V15" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W15" s="4">
-        <v>190.4</v>
-      </c>
-      <c r="X15" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y15" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z15" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA15" s="4">
-        <v>1521</v>
-      </c>
-      <c r="AB15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC15" s="3">
-        <v>0.31703999999999999</v>
-      </c>
-      <c r="AD15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE15" s="3">
-        <v>2112.66</v>
-      </c>
-      <c r="AF15" s="16">
-        <v>415.5</v>
-      </c>
-      <c r="AG15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH15" s="4" t="s">
-        <v>143</v>
-      </c>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="6"/>
+      <c r="U15" s="5"/>
+      <c r="V15" s="6"/>
+      <c r="W15" s="6"/>
+      <c r="X15" s="6"/>
+      <c r="Y15" s="6"/>
+      <c r="Z15" s="6"/>
+      <c r="AA15" s="6"/>
+      <c r="AB15" s="5"/>
+      <c r="AC15" s="5"/>
+      <c r="AD15" s="5"/>
+      <c r="AE15" s="5"/>
+      <c r="AF15" s="5"/>
+      <c r="AG15" s="5"/>
+      <c r="AH15" s="6"/>
     </row>
     <row r="16" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C16" s="10">
-        <v>800486518</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="F16" s="3">
-        <v>2024</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L16" s="4">
-        <v>36660543</v>
-      </c>
-      <c r="M16" s="3">
-        <v>46171.166666666672</v>
-      </c>
-      <c r="N16" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="O16" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="P16" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q16" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="R16" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="S16" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="T16" s="4">
-        <v>12.3</v>
-      </c>
-      <c r="U16" s="3">
-        <v>0.47</v>
-      </c>
-      <c r="V16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W16" s="4">
-        <v>71.599999999999994</v>
-      </c>
-      <c r="X16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA16" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC16" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE16" s="3">
-        <v>2689.92</v>
-      </c>
-      <c r="AF16" s="16">
-        <v>1144.7</v>
-      </c>
-      <c r="AG16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH16" s="4" t="s">
-        <v>147</v>
-      </c>
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="6"/>
+      <c r="S16" s="5"/>
+      <c r="T16" s="6"/>
+      <c r="U16" s="5"/>
+      <c r="V16" s="6"/>
+      <c r="W16" s="6"/>
+      <c r="X16" s="6"/>
+      <c r="Y16" s="6"/>
+      <c r="Z16" s="6"/>
+      <c r="AA16" s="6"/>
+      <c r="AB16" s="5"/>
+      <c r="AC16" s="5"/>
+      <c r="AD16" s="5"/>
+      <c r="AE16" s="5"/>
+      <c r="AF16" s="5"/>
+      <c r="AG16" s="5"/>
+      <c r="AH16" s="6"/>
     </row>
     <row r="17" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C17" s="10">
-        <v>800486519</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="F17" s="3">
-        <v>2024</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L17" s="4">
-        <v>35199780</v>
-      </c>
-      <c r="M17" s="3">
-        <v>45660.166666666672</v>
-      </c>
-      <c r="N17" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="O17" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="P17" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q17" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="R17" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S17" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="T17" s="4">
-        <v>12.6</v>
-      </c>
-      <c r="U17" s="3">
-        <v>0.59</v>
-      </c>
-      <c r="V17" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W17" s="4">
-        <v>186.8</v>
-      </c>
-      <c r="X17" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y17" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z17" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA17" s="4">
-        <v>1355</v>
-      </c>
-      <c r="AB17" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC17" s="3">
-        <v>0.39629999999999999</v>
-      </c>
-      <c r="AD17" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE17" s="3">
-        <v>1296.8</v>
-      </c>
-      <c r="AF17" s="16">
-        <v>541.04999999999995</v>
-      </c>
-      <c r="AG17" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH17" s="4" t="s">
-        <v>150</v>
-      </c>
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="5"/>
+      <c r="T17" s="6"/>
+      <c r="U17" s="5"/>
+      <c r="V17" s="6"/>
+      <c r="W17" s="6"/>
+      <c r="X17" s="6"/>
+      <c r="Y17" s="6"/>
+      <c r="Z17" s="6"/>
+      <c r="AA17" s="6"/>
+      <c r="AB17" s="5"/>
+      <c r="AC17" s="5"/>
+      <c r="AD17" s="5"/>
+      <c r="AE17" s="5"/>
+      <c r="AF17" s="5"/>
+      <c r="AG17" s="5"/>
+      <c r="AH17" s="6"/>
     </row>
     <row r="18" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="3">
-        <v>7265672</v>
-      </c>
-      <c r="C18" s="10">
-        <v>800486521</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="F18" s="3">
-        <v>2024</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L18" s="4">
-        <v>35199780</v>
-      </c>
-      <c r="M18" s="3">
-        <v>45660.166666666672</v>
-      </c>
-      <c r="N18" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="O18" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="P18" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q18" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="R18" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S18" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="T18" s="4">
-        <v>12.7</v>
-      </c>
-      <c r="U18" s="3">
-        <v>0.69</v>
-      </c>
-      <c r="V18" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W18" s="4">
-        <v>176</v>
-      </c>
-      <c r="X18" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y18" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z18" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA18" s="4">
-        <v>1363</v>
-      </c>
-      <c r="AB18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC18" s="3">
-        <v>0.42271999999999998</v>
-      </c>
-      <c r="AD18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE18" s="3">
-        <v>941.38</v>
-      </c>
-      <c r="AF18" s="16">
-        <v>239.3</v>
-      </c>
-      <c r="AG18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH18" s="4" t="s">
-        <v>152</v>
-      </c>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="6"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="6"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="6"/>
+      <c r="S18" s="5"/>
+      <c r="T18" s="6"/>
+      <c r="U18" s="5"/>
+      <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
+      <c r="X18" s="6"/>
+      <c r="Y18" s="6"/>
+      <c r="Z18" s="6"/>
+      <c r="AA18" s="6"/>
+      <c r="AB18" s="5"/>
+      <c r="AC18" s="5"/>
+      <c r="AD18" s="5"/>
+      <c r="AE18" s="5"/>
+      <c r="AF18" s="5"/>
+      <c r="AG18" s="5"/>
+      <c r="AH18" s="6"/>
     </row>
     <row r="19" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="8"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
       <c r="H19" s="5"/>
@@ -2800,8 +1762,8 @@
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="8"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
@@ -37680,442 +36642,10 @@
       <c r="AG988" s="5"/>
       <c r="AH988" s="6"/>
     </row>
-    <row r="989" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A989" s="5"/>
-      <c r="B989" s="5"/>
-      <c r="C989" s="5"/>
-      <c r="D989" s="5"/>
-      <c r="E989" s="5"/>
-      <c r="F989" s="5"/>
-      <c r="G989" s="5"/>
-      <c r="H989" s="5"/>
-      <c r="I989" s="5"/>
-      <c r="J989" s="5"/>
-      <c r="K989" s="5"/>
-      <c r="L989" s="6"/>
-      <c r="M989" s="5"/>
-      <c r="N989" s="6"/>
-      <c r="O989" s="6"/>
-      <c r="P989" s="6"/>
-      <c r="Q989" s="5"/>
-      <c r="R989" s="6"/>
-      <c r="S989" s="5"/>
-      <c r="T989" s="6"/>
-      <c r="U989" s="5"/>
-      <c r="V989" s="6"/>
-      <c r="W989" s="6"/>
-      <c r="X989" s="6"/>
-      <c r="Y989" s="6"/>
-      <c r="Z989" s="6"/>
-      <c r="AA989" s="6"/>
-      <c r="AB989" s="5"/>
-      <c r="AC989" s="5"/>
-      <c r="AD989" s="5"/>
-      <c r="AE989" s="5"/>
-      <c r="AF989" s="5"/>
-      <c r="AG989" s="5"/>
-      <c r="AH989" s="6"/>
-    </row>
-    <row r="990" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A990" s="5"/>
-      <c r="B990" s="5"/>
-      <c r="C990" s="5"/>
-      <c r="D990" s="5"/>
-      <c r="E990" s="5"/>
-      <c r="F990" s="5"/>
-      <c r="G990" s="5"/>
-      <c r="H990" s="5"/>
-      <c r="I990" s="5"/>
-      <c r="J990" s="5"/>
-      <c r="K990" s="5"/>
-      <c r="L990" s="6"/>
-      <c r="M990" s="5"/>
-      <c r="N990" s="6"/>
-      <c r="O990" s="6"/>
-      <c r="P990" s="6"/>
-      <c r="Q990" s="5"/>
-      <c r="R990" s="6"/>
-      <c r="S990" s="5"/>
-      <c r="T990" s="6"/>
-      <c r="U990" s="5"/>
-      <c r="V990" s="6"/>
-      <c r="W990" s="6"/>
-      <c r="X990" s="6"/>
-      <c r="Y990" s="6"/>
-      <c r="Z990" s="6"/>
-      <c r="AA990" s="6"/>
-      <c r="AB990" s="5"/>
-      <c r="AC990" s="5"/>
-      <c r="AD990" s="5"/>
-      <c r="AE990" s="5"/>
-      <c r="AF990" s="5"/>
-      <c r="AG990" s="5"/>
-      <c r="AH990" s="6"/>
-    </row>
-    <row r="991" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A991" s="5"/>
-      <c r="B991" s="5"/>
-      <c r="C991" s="5"/>
-      <c r="D991" s="5"/>
-      <c r="E991" s="5"/>
-      <c r="F991" s="5"/>
-      <c r="G991" s="5"/>
-      <c r="H991" s="5"/>
-      <c r="I991" s="5"/>
-      <c r="J991" s="5"/>
-      <c r="K991" s="5"/>
-      <c r="L991" s="6"/>
-      <c r="M991" s="5"/>
-      <c r="N991" s="6"/>
-      <c r="O991" s="6"/>
-      <c r="P991" s="6"/>
-      <c r="Q991" s="5"/>
-      <c r="R991" s="6"/>
-      <c r="S991" s="5"/>
-      <c r="T991" s="6"/>
-      <c r="U991" s="5"/>
-      <c r="V991" s="6"/>
-      <c r="W991" s="6"/>
-      <c r="X991" s="6"/>
-      <c r="Y991" s="6"/>
-      <c r="Z991" s="6"/>
-      <c r="AA991" s="6"/>
-      <c r="AB991" s="5"/>
-      <c r="AC991" s="5"/>
-      <c r="AD991" s="5"/>
-      <c r="AE991" s="5"/>
-      <c r="AF991" s="5"/>
-      <c r="AG991" s="5"/>
-      <c r="AH991" s="6"/>
-    </row>
-    <row r="992" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A992" s="5"/>
-      <c r="B992" s="5"/>
-      <c r="C992" s="5"/>
-      <c r="D992" s="5"/>
-      <c r="E992" s="5"/>
-      <c r="F992" s="5"/>
-      <c r="G992" s="5"/>
-      <c r="H992" s="5"/>
-      <c r="I992" s="5"/>
-      <c r="J992" s="5"/>
-      <c r="K992" s="5"/>
-      <c r="L992" s="6"/>
-      <c r="M992" s="5"/>
-      <c r="N992" s="6"/>
-      <c r="O992" s="6"/>
-      <c r="P992" s="6"/>
-      <c r="Q992" s="5"/>
-      <c r="R992" s="6"/>
-      <c r="S992" s="5"/>
-      <c r="T992" s="6"/>
-      <c r="U992" s="5"/>
-      <c r="V992" s="6"/>
-      <c r="W992" s="6"/>
-      <c r="X992" s="6"/>
-      <c r="Y992" s="6"/>
-      <c r="Z992" s="6"/>
-      <c r="AA992" s="6"/>
-      <c r="AB992" s="5"/>
-      <c r="AC992" s="5"/>
-      <c r="AD992" s="5"/>
-      <c r="AE992" s="5"/>
-      <c r="AF992" s="5"/>
-      <c r="AG992" s="5"/>
-      <c r="AH992" s="6"/>
-    </row>
-    <row r="993" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A993" s="5"/>
-      <c r="B993" s="5"/>
-      <c r="C993" s="5"/>
-      <c r="D993" s="5"/>
-      <c r="E993" s="5"/>
-      <c r="F993" s="5"/>
-      <c r="G993" s="5"/>
-      <c r="H993" s="5"/>
-      <c r="I993" s="5"/>
-      <c r="J993" s="5"/>
-      <c r="K993" s="5"/>
-      <c r="L993" s="6"/>
-      <c r="M993" s="5"/>
-      <c r="N993" s="6"/>
-      <c r="O993" s="6"/>
-      <c r="P993" s="6"/>
-      <c r="Q993" s="5"/>
-      <c r="R993" s="6"/>
-      <c r="S993" s="5"/>
-      <c r="T993" s="6"/>
-      <c r="U993" s="5"/>
-      <c r="V993" s="6"/>
-      <c r="W993" s="6"/>
-      <c r="X993" s="6"/>
-      <c r="Y993" s="6"/>
-      <c r="Z993" s="6"/>
-      <c r="AA993" s="6"/>
-      <c r="AB993" s="5"/>
-      <c r="AC993" s="5"/>
-      <c r="AD993" s="5"/>
-      <c r="AE993" s="5"/>
-      <c r="AF993" s="5"/>
-      <c r="AG993" s="5"/>
-      <c r="AH993" s="6"/>
-    </row>
-    <row r="994" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A994" s="5"/>
-      <c r="B994" s="5"/>
-      <c r="C994" s="5"/>
-      <c r="D994" s="5"/>
-      <c r="E994" s="5"/>
-      <c r="F994" s="5"/>
-      <c r="G994" s="5"/>
-      <c r="H994" s="5"/>
-      <c r="I994" s="5"/>
-      <c r="J994" s="5"/>
-      <c r="K994" s="5"/>
-      <c r="L994" s="6"/>
-      <c r="M994" s="5"/>
-      <c r="N994" s="6"/>
-      <c r="O994" s="6"/>
-      <c r="P994" s="6"/>
-      <c r="Q994" s="5"/>
-      <c r="R994" s="6"/>
-      <c r="S994" s="5"/>
-      <c r="T994" s="6"/>
-      <c r="U994" s="5"/>
-      <c r="V994" s="6"/>
-      <c r="W994" s="6"/>
-      <c r="X994" s="6"/>
-      <c r="Y994" s="6"/>
-      <c r="Z994" s="6"/>
-      <c r="AA994" s="6"/>
-      <c r="AB994" s="5"/>
-      <c r="AC994" s="5"/>
-      <c r="AD994" s="5"/>
-      <c r="AE994" s="5"/>
-      <c r="AF994" s="5"/>
-      <c r="AG994" s="5"/>
-      <c r="AH994" s="6"/>
-    </row>
-    <row r="995" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A995" s="5"/>
-      <c r="B995" s="5"/>
-      <c r="C995" s="5"/>
-      <c r="D995" s="5"/>
-      <c r="E995" s="5"/>
-      <c r="F995" s="5"/>
-      <c r="G995" s="5"/>
-      <c r="H995" s="5"/>
-      <c r="I995" s="5"/>
-      <c r="J995" s="5"/>
-      <c r="K995" s="5"/>
-      <c r="L995" s="6"/>
-      <c r="M995" s="5"/>
-      <c r="N995" s="6"/>
-      <c r="O995" s="6"/>
-      <c r="P995" s="6"/>
-      <c r="Q995" s="5"/>
-      <c r="R995" s="6"/>
-      <c r="S995" s="5"/>
-      <c r="T995" s="6"/>
-      <c r="U995" s="5"/>
-      <c r="V995" s="6"/>
-      <c r="W995" s="6"/>
-      <c r="X995" s="6"/>
-      <c r="Y995" s="6"/>
-      <c r="Z995" s="6"/>
-      <c r="AA995" s="6"/>
-      <c r="AB995" s="5"/>
-      <c r="AC995" s="5"/>
-      <c r="AD995" s="5"/>
-      <c r="AE995" s="5"/>
-      <c r="AF995" s="5"/>
-      <c r="AG995" s="5"/>
-      <c r="AH995" s="6"/>
-    </row>
-    <row r="996" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A996" s="5"/>
-      <c r="B996" s="5"/>
-      <c r="C996" s="5"/>
-      <c r="D996" s="5"/>
-      <c r="E996" s="5"/>
-      <c r="F996" s="5"/>
-      <c r="G996" s="5"/>
-      <c r="H996" s="5"/>
-      <c r="I996" s="5"/>
-      <c r="J996" s="5"/>
-      <c r="K996" s="5"/>
-      <c r="L996" s="6"/>
-      <c r="M996" s="5"/>
-      <c r="N996" s="6"/>
-      <c r="O996" s="6"/>
-      <c r="P996" s="6"/>
-      <c r="Q996" s="5"/>
-      <c r="R996" s="6"/>
-      <c r="S996" s="5"/>
-      <c r="T996" s="6"/>
-      <c r="U996" s="5"/>
-      <c r="V996" s="6"/>
-      <c r="W996" s="6"/>
-      <c r="X996" s="6"/>
-      <c r="Y996" s="6"/>
-      <c r="Z996" s="6"/>
-      <c r="AA996" s="6"/>
-      <c r="AB996" s="5"/>
-      <c r="AC996" s="5"/>
-      <c r="AD996" s="5"/>
-      <c r="AE996" s="5"/>
-      <c r="AF996" s="5"/>
-      <c r="AG996" s="5"/>
-      <c r="AH996" s="6"/>
-    </row>
-    <row r="997" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A997" s="5"/>
-      <c r="B997" s="5"/>
-      <c r="C997" s="5"/>
-      <c r="D997" s="5"/>
-      <c r="E997" s="5"/>
-      <c r="F997" s="5"/>
-      <c r="G997" s="5"/>
-      <c r="H997" s="5"/>
-      <c r="I997" s="5"/>
-      <c r="J997" s="5"/>
-      <c r="K997" s="5"/>
-      <c r="L997" s="6"/>
-      <c r="M997" s="5"/>
-      <c r="N997" s="6"/>
-      <c r="O997" s="6"/>
-      <c r="P997" s="6"/>
-      <c r="Q997" s="5"/>
-      <c r="R997" s="6"/>
-      <c r="S997" s="5"/>
-      <c r="T997" s="6"/>
-      <c r="U997" s="5"/>
-      <c r="V997" s="6"/>
-      <c r="W997" s="6"/>
-      <c r="X997" s="6"/>
-      <c r="Y997" s="6"/>
-      <c r="Z997" s="6"/>
-      <c r="AA997" s="6"/>
-      <c r="AB997" s="5"/>
-      <c r="AC997" s="5"/>
-      <c r="AD997" s="5"/>
-      <c r="AE997" s="5"/>
-      <c r="AF997" s="5"/>
-      <c r="AG997" s="5"/>
-      <c r="AH997" s="6"/>
-    </row>
-    <row r="998" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A998" s="5"/>
-      <c r="B998" s="5"/>
-      <c r="C998" s="5"/>
-      <c r="D998" s="5"/>
-      <c r="E998" s="5"/>
-      <c r="F998" s="5"/>
-      <c r="G998" s="5"/>
-      <c r="H998" s="5"/>
-      <c r="I998" s="5"/>
-      <c r="J998" s="5"/>
-      <c r="K998" s="5"/>
-      <c r="L998" s="6"/>
-      <c r="M998" s="5"/>
-      <c r="N998" s="6"/>
-      <c r="O998" s="6"/>
-      <c r="P998" s="6"/>
-      <c r="Q998" s="5"/>
-      <c r="R998" s="6"/>
-      <c r="S998" s="5"/>
-      <c r="T998" s="6"/>
-      <c r="U998" s="5"/>
-      <c r="V998" s="6"/>
-      <c r="W998" s="6"/>
-      <c r="X998" s="6"/>
-      <c r="Y998" s="6"/>
-      <c r="Z998" s="6"/>
-      <c r="AA998" s="6"/>
-      <c r="AB998" s="5"/>
-      <c r="AC998" s="5"/>
-      <c r="AD998" s="5"/>
-      <c r="AE998" s="5"/>
-      <c r="AF998" s="5"/>
-      <c r="AG998" s="5"/>
-      <c r="AH998" s="6"/>
-    </row>
-    <row r="999" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A999" s="5"/>
-      <c r="B999" s="5"/>
-      <c r="C999" s="5"/>
-      <c r="D999" s="5"/>
-      <c r="E999" s="5"/>
-      <c r="F999" s="5"/>
-      <c r="G999" s="5"/>
-      <c r="H999" s="5"/>
-      <c r="I999" s="5"/>
-      <c r="J999" s="5"/>
-      <c r="K999" s="5"/>
-      <c r="L999" s="6"/>
-      <c r="M999" s="5"/>
-      <c r="N999" s="6"/>
-      <c r="O999" s="6"/>
-      <c r="P999" s="6"/>
-      <c r="Q999" s="5"/>
-      <c r="R999" s="6"/>
-      <c r="S999" s="5"/>
-      <c r="T999" s="6"/>
-      <c r="U999" s="5"/>
-      <c r="V999" s="6"/>
-      <c r="W999" s="6"/>
-      <c r="X999" s="6"/>
-      <c r="Y999" s="6"/>
-      <c r="Z999" s="6"/>
-      <c r="AA999" s="6"/>
-      <c r="AB999" s="5"/>
-      <c r="AC999" s="5"/>
-      <c r="AD999" s="5"/>
-      <c r="AE999" s="5"/>
-      <c r="AF999" s="5"/>
-      <c r="AG999" s="5"/>
-      <c r="AH999" s="6"/>
-    </row>
-    <row r="1000" spans="1:34" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1000" s="5"/>
-      <c r="B1000" s="5"/>
-      <c r="C1000" s="5"/>
-      <c r="D1000" s="5"/>
-      <c r="E1000" s="5"/>
-      <c r="F1000" s="5"/>
-      <c r="G1000" s="5"/>
-      <c r="H1000" s="5"/>
-      <c r="I1000" s="5"/>
-      <c r="J1000" s="5"/>
-      <c r="K1000" s="5"/>
-      <c r="L1000" s="6"/>
-      <c r="M1000" s="5"/>
-      <c r="N1000" s="6"/>
-      <c r="O1000" s="6"/>
-      <c r="P1000" s="6"/>
-      <c r="Q1000" s="5"/>
-      <c r="R1000" s="6"/>
-      <c r="S1000" s="5"/>
-      <c r="T1000" s="6"/>
-      <c r="U1000" s="5"/>
-      <c r="V1000" s="6"/>
-      <c r="W1000" s="6"/>
-      <c r="X1000" s="6"/>
-      <c r="Y1000" s="6"/>
-      <c r="Z1000" s="6"/>
-      <c r="AA1000" s="6"/>
-      <c r="AB1000" s="5"/>
-      <c r="AC1000" s="5"/>
-      <c r="AD1000" s="5"/>
-      <c r="AE1000" s="5"/>
-      <c r="AF1000" s="5"/>
-      <c r="AG1000" s="5"/>
-      <c r="AH1000" s="6"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>